<commit_message>
Fixed date format on a few drafts, generated test draft_input.json from LUA, started new record from json, updated bracket LUA to functional(?) export
</commit_message>
<xml_diff>
--- a/input/xlsx/103.xlsx
+++ b/input/xlsx/103.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
   <workbookPr defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Draft" sheetId="1" r:id="rId1"/>
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="559" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="560" uniqueCount="195">
   <si>
     <t>Nenni</t>
   </si>
@@ -599,6 +599,9 @@
   </si>
   <si>
     <t>Rona, Herald of Invasion // Rona, Tolarian Obliterator</t>
+  </si>
+  <si>
+    <t>07/03/2025</t>
   </si>
 </sst>
 </file>
@@ -664,7 +667,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -681,7 +684,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2893,12 +2895,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" s="6">
-        <v>45841</v>
+      <c r="A1" s="6" t="s">
+        <v>194</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="6" t="s">
         <v>192</v>
       </c>
     </row>

</xml_diff>